<commit_message>
começando modelo lógico, testando funções no modelo físico
</commit_message>
<xml_diff>
--- a/Documentos/modelo_dicionario_de_dados.xlsx
+++ b/Documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="150">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -157,6 +157,12 @@
   </si>
   <si>
     <t xml:space="preserve">identifica o funcionário que registrou o cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">identifica o cargo do funcionário que registrou o cliente</t>
   </si>
   <si>
     <r>
@@ -181,6 +187,9 @@
     <t xml:space="preserve">cpf</t>
   </si>
   <si>
+    <t xml:space="preserve">UNIQUE</t>
+  </si>
+  <si>
     <t xml:space="preserve">identifica o funcionario pelo cpf</t>
   </si>
   <si>
@@ -211,6 +220,12 @@
     <t xml:space="preserve">Nome da situação</t>
   </si>
   <si>
+    <t xml:space="preserve">Identifica quando a situação foi criada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identifica se a situação está ativa</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chave primária de identificação do cargo</t>
   </si>
   <si>
@@ -220,30 +235,74 @@
     <t xml:space="preserve">Campo da data de registro do equipamento</t>
   </si>
   <si>
+    <t xml:space="preserve">id_marca</t>
+  </si>
+  <si>
     <t xml:space="preserve">marca</t>
   </si>
   <si>
     <t xml:space="preserve">Identifica a marca do aparelho</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Consolas"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">id_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Consolas"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">modelo</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">modelo</t>
   </si>
   <si>
     <t xml:space="preserve">Identifica a modelo do aparelho</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Consolas"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">id_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Consolas"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">tipo</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">tipo</t>
   </si>
   <si>
     <t xml:space="preserve">Identifica a tipo do aparelho</t>
   </si>
   <si>
+    <t xml:space="preserve">serial_number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">identifica o numero de serie do aparelho</t>
+  </si>
+  <si>
     <t xml:space="preserve">imei</t>
   </si>
   <si>
-    <t xml:space="preserve">UNIQUE</t>
-  </si>
-  <si>
     <t xml:space="preserve">identifica o imei do aparelho</t>
   </si>
   <si>
@@ -256,7 +315,22 @@
     <t xml:space="preserve">identifica a que ordem de serviço ele pertence</t>
   </si>
   <si>
-    <t xml:space="preserve">funcionario_equipamento</t>
+    <t xml:space="preserve">Chave primária de identificação da marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">identifica o cargo do funcionário que registrou a marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária de identificação da modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">identifica o cargo do funcionário que registrou a modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária de identificação da tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">identifica o cargo do funcionário que registrou a tipo</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -455,7 +529,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -527,6 +601,11 @@
       <family val="0"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Consolas"/>
+      <family val="0"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="13"/>
       <color rgb="FF1E3A8A"/>
@@ -535,7 +614,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -552,6 +631,54 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF8FAFC"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E8FC"/>
+        <bgColor rgb="FFD5E8D4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE1D5E7"/>
+        <bgColor rgb="FFCBD5E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD5E8D4"/>
+        <bgColor rgb="FFD9E8FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8CECC"/>
+        <bgColor rgb="FFE1D5E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF99CC"/>
+        <bgColor rgb="FFCC99FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0080"/>
+        <bgColor rgb="FFFF00FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF66B3"/>
+        <bgColor rgb="FFFF99CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -604,7 +731,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="61">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -669,8 +796,172 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -681,7 +972,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -702,7 +993,7 @@
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFF0080"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
@@ -710,14 +1001,14 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFE1D5E7"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF8FAFC"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFFFF2CC"/>
+      <rgbColor rgb="FFD9E8FC"/>
       <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FFFF66B3"/>
       <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFCBD5E1"/>
       <rgbColor rgb="FF000080"/>
@@ -729,13 +1020,13 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFF8FAFC"/>
+      <rgbColor rgb="FFD5E8D4"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFF8CECC"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -937,7 +1228,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1048576"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.79"/>
@@ -1166,122 +1457,122 @@
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
     </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
+    <row r="17" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10" t="s">
+      <c r="C17" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" s="9" t="s">
+      <c r="F17" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="H17" s="9"/>
-      <c r="I17" s="11" t="s">
+      <c r="H17" s="17"/>
+      <c r="I17" s="19" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
+    <row r="18" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="15" t="s">
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="19" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
+    <row r="19" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G19" s="9" t="s">
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="H19" s="9"/>
-      <c r="I19" s="11" t="s">
+      <c r="H19" s="17"/>
+      <c r="I19" s="19" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
+    <row r="20" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14" t="s">
+      <c r="C20" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="F20" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="13" t="s">
+      <c r="F20" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="H20" s="13" t="s">
+      <c r="H20" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="I20" s="15" t="s">
+      <c r="I20" s="19" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
+    <row r="21" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G21" s="9" t="n">
+      <c r="C21" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="9"/>
-      <c r="I21" s="11" t="s">
+      <c r="H21" s="17"/>
+      <c r="I21" s="19" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1296,633 +1587,749 @@
       <c r="H22" s="13"/>
       <c r="I22" s="15"/>
     </row>
-    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
+    <row r="23" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10" t="s">
+      <c r="C23" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="9" t="s">
+      <c r="F23" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="H23" s="9"/>
-      <c r="I23" s="11" t="s">
+      <c r="H23" s="22"/>
+      <c r="I23" s="24" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
+    <row r="24" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="15" t="s">
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="24" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12" t="s">
+    <row r="25" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="11" t="s">
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="24" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="s">
+    <row r="26" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C26" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10" t="s">
+      <c r="C26" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="23"/>
+      <c r="E26" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="F26" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9" t="s">
+      <c r="F26" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="I26" s="11" t="s">
+      <c r="I26" s="24" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="s">
+    <row r="27" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27" s="24" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G27" s="9" t="n">
+      <c r="C28" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G28" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="9"/>
-      <c r="I27" s="11" t="s">
+      <c r="H28" s="22"/>
+      <c r="I28" s="24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="H29" s="22"/>
+      <c r="I29" s="24" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="I30" s="24" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="I31" s="24" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="11"/>
+    </row>
+    <row r="33" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B33" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="H33" s="27"/>
+      <c r="I33" s="29" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="34" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="D34" s="28"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
+      <c r="I34" s="29" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C35" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G35" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="H35" s="27"/>
+      <c r="I35" s="29" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C36" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="28"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="27"/>
+      <c r="H36" s="27"/>
+      <c r="I36" s="29" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="13"/>
+      <c r="H37" s="13"/>
+      <c r="I37" s="15"/>
+    </row>
+    <row r="38" s="35" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38" s="31" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="33"/>
+      <c r="E38" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="F38" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G38" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="H38" s="32"/>
+      <c r="I38" s="34" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="39" s="35" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C39" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="D39" s="33"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="H39" s="32"/>
+      <c r="I39" s="34" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="40" s="35" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="C40" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="33"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="32"/>
+      <c r="I40" s="34" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="14"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="15"/>
+    </row>
+    <row r="42" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B42" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="C42" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D42" s="38"/>
+      <c r="E42" s="38" t="s">
+        <v>20</v>
+      </c>
+      <c r="F42" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G42" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="H42" s="37"/>
+      <c r="I42" s="39" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="43" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B43" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="C43" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="G43" s="37"/>
+      <c r="H43" s="37"/>
+      <c r="I43" s="39" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="44" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B44" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="C44" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G44" s="37"/>
+      <c r="H44" s="37"/>
+      <c r="I44" s="39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B45" s="36" t="s">
+        <v>65</v>
+      </c>
+      <c r="C45" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="38"/>
+      <c r="E45" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="F45" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G45" s="37"/>
+      <c r="H45" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="I45" s="39" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="46" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B46" s="41" t="s">
+        <v>68</v>
+      </c>
+      <c r="C46" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D46" s="38"/>
+      <c r="E46" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="F46" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G46" s="37"/>
+      <c r="H46" s="37" t="s">
+        <v>69</v>
+      </c>
+      <c r="I46" s="39" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="47" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B47" s="41" t="s">
+        <v>71</v>
+      </c>
+      <c r="C47" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D47" s="38"/>
+      <c r="E47" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="F47" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="G47" s="37"/>
+      <c r="H47" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="I47" s="39" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="48" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B48" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="C48" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D48" s="38"/>
+      <c r="E48" s="38"/>
+      <c r="F48" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="G48" s="37" t="s">
+        <v>49</v>
+      </c>
+      <c r="H48" s="37"/>
+      <c r="I48" s="39" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="49" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B49" s="36" t="s">
+        <v>76</v>
+      </c>
+      <c r="C49" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D49" s="38"/>
+      <c r="E49" s="38"/>
+      <c r="F49" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="G49" s="37" t="s">
+        <v>49</v>
+      </c>
+      <c r="H49" s="37"/>
+      <c r="I49" s="39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="50" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B50" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="C50" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D50" s="38"/>
+      <c r="E50" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="F50" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G50" s="37"/>
+      <c r="H50" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="I50" s="39" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="8"/>
+      <c r="B51" s="12"/>
+      <c r="C51" s="13"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="14"/>
+      <c r="F51" s="14"/>
+      <c r="G51" s="13"/>
+      <c r="H51" s="13"/>
+      <c r="I51" s="15"/>
+    </row>
+    <row r="52" s="47" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="B52" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="C52" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="D52" s="45"/>
+      <c r="E52" s="45" t="s">
+        <v>20</v>
+      </c>
+      <c r="F52" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="G52" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="H52" s="44"/>
+      <c r="I52" s="46" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="53" s="47" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="B53" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="C53" s="44" t="s">
+        <v>25</v>
+      </c>
+      <c r="D53" s="45"/>
+      <c r="E53" s="45"/>
+      <c r="F53" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="G53" s="44" t="s">
+        <v>49</v>
+      </c>
+      <c r="H53" s="44"/>
+      <c r="I53" s="46" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="54" s="47" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="B54" s="43" t="s">
+        <v>41</v>
+      </c>
+      <c r="C54" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="D54" s="45"/>
+      <c r="E54" s="45"/>
+      <c r="F54" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="G54" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" s="44"/>
+      <c r="I54" s="46" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="55" s="47" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="B55" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="C55" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="D55" s="45"/>
+      <c r="E55" s="45" t="s">
+        <v>37</v>
+      </c>
+      <c r="F55" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="G55" s="44"/>
+      <c r="H55" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="I55" s="46" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="56" s="47" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" s="43" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8"/>
-      <c r="B31" s="8"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="11"/>
-    </row>
-    <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F32" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="H32" s="9"/>
-      <c r="I32" s="11" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G33" s="9"/>
-      <c r="H33" s="9"/>
-      <c r="I33" s="11" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="15"/>
-    </row>
-    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F35" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G35" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="H35" s="9"/>
-      <c r="I35" s="11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="11" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G37" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" s="9"/>
-      <c r="I37" s="11" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="15"/>
-    </row>
-    <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F39" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G39" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="H39" s="9"/>
-      <c r="I39" s="11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="11" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C41" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
-      <c r="F41" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G41" s="9"/>
-      <c r="H41" s="9"/>
-      <c r="I41" s="11" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14" t="s">
+      <c r="C56" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="D56" s="45"/>
+      <c r="E56" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="F42" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G42" s="13"/>
-      <c r="H42" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="I42" s="15" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="F43" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G43" s="13"/>
-      <c r="H43" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="I43" s="15" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="F44" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="G44" s="13"/>
-      <c r="H44" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="I44" s="15" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="C45" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="G45" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="H45" s="13"/>
-      <c r="I45" s="15" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B46" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="C46" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="F46" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G46" s="13"/>
-      <c r="H46" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="I46" s="15" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="8"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="13"/>
-      <c r="H47" s="13"/>
-      <c r="I47" s="15"/>
-    </row>
-    <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="8"/>
-      <c r="B48" s="12"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="13"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="15"/>
-    </row>
-    <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="8"/>
-      <c r="B49" s="12"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="13"/>
-      <c r="H49" s="13"/>
-      <c r="I49" s="15"/>
-    </row>
-    <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="8"/>
-      <c r="B50" s="8"/>
-      <c r="C50" s="9"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
-      <c r="G50" s="9"/>
-      <c r="H50" s="9"/>
-      <c r="I50" s="11"/>
-    </row>
-    <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B51" s="8"/>
-      <c r="C51" s="9"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
-      <c r="F51" s="10"/>
-      <c r="G51" s="9"/>
-      <c r="H51" s="9"/>
-      <c r="I51" s="11"/>
-    </row>
-    <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="12"/>
-      <c r="B52" s="12"/>
-      <c r="C52" s="13"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="13"/>
-      <c r="H52" s="13"/>
-      <c r="I52" s="15"/>
-    </row>
-    <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="8"/>
-      <c r="B53" s="8"/>
-      <c r="C53" s="9"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="10"/>
-      <c r="F53" s="10"/>
-      <c r="G53" s="9"/>
-      <c r="H53" s="9"/>
-      <c r="I53" s="11"/>
-    </row>
-    <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="12"/>
-      <c r="B54" s="12"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="13"/>
-      <c r="H54" s="13"/>
-      <c r="I54" s="15"/>
-    </row>
-    <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="8"/>
-      <c r="B55" s="8"/>
-      <c r="C55" s="9"/>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
-      <c r="F55" s="10"/>
-      <c r="G55" s="9"/>
-      <c r="H55" s="9"/>
-      <c r="I55" s="11"/>
-    </row>
-    <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="12"/>
-      <c r="B56" s="12"/>
-      <c r="C56" s="13"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
-      <c r="F56" s="14"/>
-      <c r="G56" s="13"/>
-      <c r="H56" s="13"/>
-      <c r="I56" s="15"/>
+      <c r="F56" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="G56" s="44"/>
+      <c r="H56" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="I56" s="46" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="8"/>
@@ -1935,60 +2342,126 @@
       <c r="H57" s="9"/>
       <c r="I57" s="11"/>
     </row>
-    <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="12"/>
-      <c r="B58" s="12"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="13"/>
-      <c r="H58" s="13"/>
-      <c r="I58" s="15"/>
-    </row>
-    <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="8"/>
-      <c r="B59" s="8"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
-      <c r="G59" s="9"/>
-      <c r="H59" s="9"/>
-      <c r="I59" s="11"/>
-    </row>
-    <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="12"/>
-      <c r="B60" s="12"/>
-      <c r="C60" s="13"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="14"/>
-      <c r="F60" s="14"/>
-      <c r="G60" s="13"/>
-      <c r="H60" s="13"/>
-      <c r="I60" s="15"/>
-    </row>
-    <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="8"/>
-      <c r="B61" s="8"/>
-      <c r="C61" s="9"/>
-      <c r="D61" s="10"/>
-      <c r="E61" s="10"/>
-      <c r="F61" s="10"/>
-      <c r="G61" s="9"/>
-      <c r="H61" s="9"/>
-      <c r="I61" s="11"/>
-    </row>
-    <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="12"/>
-      <c r="B62" s="12"/>
-      <c r="C62" s="13"/>
-      <c r="D62" s="14"/>
-      <c r="E62" s="14"/>
-      <c r="F62" s="14"/>
-      <c r="G62" s="13"/>
-      <c r="H62" s="13"/>
-      <c r="I62" s="15"/>
+    <row r="58" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="B58" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="C58" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="D58" s="50"/>
+      <c r="E58" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="F58" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="G58" s="49" t="s">
+        <v>22</v>
+      </c>
+      <c r="H58" s="49"/>
+      <c r="I58" s="51" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="59" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="B59" s="48" t="s">
+        <v>24</v>
+      </c>
+      <c r="C59" s="49" t="s">
+        <v>25</v>
+      </c>
+      <c r="D59" s="50"/>
+      <c r="E59" s="50"/>
+      <c r="F59" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="G59" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="H59" s="49"/>
+      <c r="I59" s="51" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="60" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="B60" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="C60" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="D60" s="50"/>
+      <c r="E60" s="50"/>
+      <c r="F60" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="G60" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" s="49"/>
+      <c r="I60" s="51" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="61" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="B61" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C61" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="D61" s="50"/>
+      <c r="E61" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="F61" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="G61" s="49"/>
+      <c r="H61" s="49" t="s">
+        <v>17</v>
+      </c>
+      <c r="I61" s="51" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="62" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="B62" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="C62" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="D62" s="50"/>
+      <c r="E62" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="F62" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="G62" s="49"/>
+      <c r="H62" s="49" t="s">
+        <v>17</v>
+      </c>
+      <c r="I62" s="51" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="8"/>
@@ -2001,73 +2474,182 @@
       <c r="H63" s="9"/>
       <c r="I63" s="11"/>
     </row>
-    <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="12"/>
-      <c r="B64" s="12"/>
-      <c r="C64" s="13"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="14"/>
-      <c r="F64" s="14"/>
-      <c r="G64" s="13"/>
-      <c r="H64" s="13"/>
-      <c r="I64" s="15"/>
-    </row>
-    <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="8"/>
-      <c r="B65" s="8"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="10"/>
-      <c r="E65" s="10"/>
-      <c r="F65" s="10"/>
-      <c r="G65" s="9"/>
-      <c r="H65" s="9"/>
-      <c r="I65" s="11"/>
-    </row>
-    <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="12"/>
-      <c r="B66" s="12"/>
-      <c r="C66" s="13"/>
-      <c r="D66" s="14"/>
-      <c r="E66" s="14"/>
-      <c r="F66" s="14"/>
-      <c r="G66" s="13"/>
-      <c r="H66" s="13"/>
-      <c r="I66" s="15"/>
-    </row>
-    <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="8"/>
-      <c r="B67" s="8"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="10"/>
-      <c r="E67" s="10"/>
-      <c r="F67" s="10"/>
-      <c r="G67" s="9"/>
-      <c r="H67" s="9"/>
-      <c r="I67" s="11"/>
-    </row>
-    <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="12"/>
-      <c r="B68" s="12"/>
-      <c r="C68" s="13"/>
-      <c r="D68" s="14"/>
-      <c r="E68" s="14"/>
-      <c r="F68" s="14"/>
-      <c r="G68" s="13"/>
-      <c r="H68" s="13"/>
-      <c r="I68" s="15"/>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="64" s="57" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="53" t="s">
+        <v>72</v>
+      </c>
+      <c r="B64" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="C64" s="54" t="s">
+        <v>19</v>
+      </c>
+      <c r="D64" s="55"/>
+      <c r="E64" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="F64" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="G64" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="H64" s="54"/>
+      <c r="I64" s="56" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="65" s="57" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="53" t="s">
+        <v>72</v>
+      </c>
+      <c r="B65" s="53" t="s">
+        <v>24</v>
+      </c>
+      <c r="C65" s="54" t="s">
+        <v>25</v>
+      </c>
+      <c r="D65" s="55"/>
+      <c r="E65" s="55"/>
+      <c r="F65" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="G65" s="54" t="s">
+        <v>49</v>
+      </c>
+      <c r="H65" s="54"/>
+      <c r="I65" s="56" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="66" s="57" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="53" t="s">
+        <v>72</v>
+      </c>
+      <c r="B66" s="53" t="s">
+        <v>41</v>
+      </c>
+      <c r="C66" s="54" t="s">
+        <v>19</v>
+      </c>
+      <c r="D66" s="55"/>
+      <c r="E66" s="55"/>
+      <c r="F66" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="G66" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" s="54"/>
+      <c r="I66" s="56" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="67" s="57" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="53" t="s">
+        <v>72</v>
+      </c>
+      <c r="B67" s="53" t="s">
+        <v>43</v>
+      </c>
+      <c r="C67" s="54" t="s">
+        <v>19</v>
+      </c>
+      <c r="D67" s="55"/>
+      <c r="E67" s="55" t="s">
+        <v>37</v>
+      </c>
+      <c r="F67" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="G67" s="54"/>
+      <c r="H67" s="54" t="s">
+        <v>17</v>
+      </c>
+      <c r="I67" s="56" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="68" s="57" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="53" t="s">
+        <v>72</v>
+      </c>
+      <c r="B68" s="53" t="s">
+        <v>45</v>
+      </c>
+      <c r="C68" s="54" t="s">
+        <v>19</v>
+      </c>
+      <c r="D68" s="55"/>
+      <c r="E68" s="55" t="s">
+        <v>37</v>
+      </c>
+      <c r="F68" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="G68" s="54"/>
+      <c r="H68" s="54" t="s">
+        <v>17</v>
+      </c>
+      <c r="I68" s="56" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="8"/>
+      <c r="B69" s="8"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="10"/>
+      <c r="E69" s="10"/>
+      <c r="F69" s="10"/>
+      <c r="G69" s="9"/>
+      <c r="H69" s="9"/>
+      <c r="I69" s="11"/>
+    </row>
+    <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="12"/>
+      <c r="B70" s="12"/>
+      <c r="C70" s="13"/>
+      <c r="D70" s="14"/>
+      <c r="E70" s="14"/>
+      <c r="F70" s="14"/>
+      <c r="G70" s="13"/>
+      <c r="H70" s="13"/>
+      <c r="I70" s="15"/>
+    </row>
+    <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="8"/>
+      <c r="B71" s="8"/>
+      <c r="C71" s="9"/>
+      <c r="D71" s="10"/>
+      <c r="E71" s="10"/>
+      <c r="F71" s="10"/>
+      <c r="G71" s="9"/>
+      <c r="H71" s="9"/>
+      <c r="I71" s="11"/>
+    </row>
+    <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="12"/>
+      <c r="B72" s="12"/>
+      <c r="C72" s="13"/>
+      <c r="D72" s="14"/>
+      <c r="E72" s="14"/>
+      <c r="F72" s="14"/>
+      <c r="G72" s="13"/>
+      <c r="H72" s="13"/>
+      <c r="I72" s="15"/>
+    </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C15 C17:C68" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C15 C17:C72" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E15 E17:E68" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E15 E17:E72" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F15 F17:F68" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F15 F17:F72" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2102,89 +2684,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>76</v>
+      <c r="A4" s="58" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="59" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>78</v>
+      <c r="A5" s="58" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="59" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>80</v>
+      <c r="A6" s="58" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="59" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>82</v>
+      <c r="A7" s="58" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" s="59" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>84</v>
+      <c r="A8" s="58" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="59" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>86</v>
+      <c r="A9" s="58" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="59" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>88</v>
+      <c r="A10" s="58" t="s">
+        <v>101</v>
+      </c>
+      <c r="B10" s="59" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>90</v>
+      <c r="A11" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" s="59" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>92</v>
+      <c r="A12" s="58" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="59" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
-        <v>93</v>
+      <c r="A14" s="60" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2192,7 +2774,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>10</v>
@@ -2207,10 +2789,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>16</v>
@@ -2218,16 +2800,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>20</v>
@@ -2236,131 +2818,131 @@
         <v>21</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="H17" s="12" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>21</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>21</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>21</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>37</v>
@@ -2369,27 +2951,27 @@
         <v>21</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>20</v>
@@ -2398,65 +2980,65 @@
         <v>21</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C24" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="D24" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="E24" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="C24" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>106</v>
-      </c>
       <c r="F24" s="10" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -2486,12 +3068,12 @@
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>37</v>
@@ -2502,23 +3084,23 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2528,27 +3110,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
seguindo para o módulo B - categorias, ordem de serviço, peças e serviços
</commit_message>
<xml_diff>
--- a/Documentos/modelo_dicionario_de_dados.xlsx
+++ b/Documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="174">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -162,26 +162,13 @@
     <t xml:space="preserve">id_funcionario_cargo</t>
   </si>
   <si>
+    <t xml:space="preserve">CHECK(1,2)</t>
+  </si>
+  <si>
     <t xml:space="preserve">identifica o cargo do funcionário que registrou o cliente</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Campo para identificar a situação do cliente </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">(0 ou 1)</t>
-    </r>
+    <t xml:space="preserve">Campo para identificar a situação do cliente (0 ou 1)</t>
   </si>
   <si>
     <t xml:space="preserve">cpf</t>
@@ -244,23 +231,7 @@
     <t xml:space="preserve">Identifica a marca do aparelho</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Consolas"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">id_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Consolas"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">modelo</t>
-    </r>
+    <t xml:space="preserve">id_modelo</t>
   </si>
   <si>
     <t xml:space="preserve">modelo</t>
@@ -269,23 +240,7 @@
     <t xml:space="preserve">Identifica a modelo do aparelho</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Consolas"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">id_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Consolas"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">tipo</t>
-    </r>
+    <t xml:space="preserve">id_tipo</t>
   </si>
   <si>
     <t xml:space="preserve">tipo</t>
@@ -331,6 +286,75 @@
   </si>
   <si>
     <t xml:space="preserve">identifica o cargo do funcionário que registrou a tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Default</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referência</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordem_Servico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">equipamento(id)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funcionario(id)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_cargo_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funcionario(id, id_cargo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATETIME('now','localtime')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_fechamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">defeito_relatado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">relatorio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">status_atual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">situacao(nome)*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor_total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tecnico_abertura</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -529,13 +553,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -555,45 +578,42 @@
     <font>
       <b val="true"/>
       <sz val="16"/>
-      <color rgb="FF1E3A8A"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
       <sz val="11"/>
-      <color rgb="FF475569"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
       <name val="Consolas"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -607,14 +627,20 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="13"/>
-      <color rgb="FF1E3A8A"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -666,7 +692,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF99CC"/>
-        <bgColor rgb="FFCC99FF"/>
+        <bgColor rgb="FFCB99FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -679,6 +705,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFF66B3"/>
         <bgColor rgb="FFFF99CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCB99FF"/>
+        <bgColor rgb="FF9999FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -731,7 +763,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="69">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -836,6 +868,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -876,6 +912,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -900,10 +940,6 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -924,6 +960,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -944,6 +984,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -964,6 +1008,26 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -972,7 +1036,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1025,7 +1089,7 @@
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFCB99FF"/>
       <rgbColor rgb="FFF8CECC"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
@@ -1091,14 +1155,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1106,58 +1170,25 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1175,48 +1206,12 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -1228,15 +1223,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
-  <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:I81"/>
+  <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="35.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="2" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="35.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="52.87"/>
   </cols>
@@ -1246,24 +1241,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="6"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="6"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
@@ -1271,7 +1266,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
@@ -1449,15 +1444,15 @@
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12"/>
       <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
       <c r="I16" s="12"/>
     </row>
-    <row r="17" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" s="20" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
         <v>17</v>
       </c>
@@ -1482,7 +1477,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" s="20" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
         <v>17</v>
       </c>
@@ -1503,7 +1498,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" s="20" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
         <v>17</v>
       </c>
@@ -1526,7 +1521,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" s="20" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
         <v>17</v>
       </c>
@@ -1553,7 +1548,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" s="20" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
         <v>17</v>
       </c>
@@ -1576,7 +1571,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12"/>
       <c r="B22" s="12"/>
       <c r="C22" s="13"/>
@@ -1587,7 +1582,7 @@
       <c r="H22" s="13"/>
       <c r="I22" s="15"/>
     </row>
-    <row r="23" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" s="25" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
         <v>27</v>
       </c>
@@ -1612,7 +1607,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" s="25" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
         <v>27</v>
       </c>
@@ -1633,7 +1628,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" s="25" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
         <v>27</v>
       </c>
@@ -1654,7 +1649,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" s="25" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
         <v>27</v>
       </c>
@@ -1679,7 +1674,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="27" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" s="25" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
         <v>27</v>
       </c>
@@ -1696,15 +1691,17 @@
       <c r="F27" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="G27" s="22"/>
+      <c r="G27" s="22" t="s">
+        <v>46</v>
+      </c>
       <c r="H27" s="22" t="s">
         <v>17</v>
       </c>
       <c r="I27" s="24" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="28" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" s="25" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
         <v>27</v>
       </c>
@@ -1723,16 +1720,16 @@
         <v>1</v>
       </c>
       <c r="H28" s="22"/>
-      <c r="I28" s="24" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="29" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I28" s="26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" s="25" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C29" s="22" t="s">
         <v>25</v>
@@ -1743,19 +1740,19 @@
         <v>21</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H29" s="22"/>
       <c r="I29" s="24" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="30" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" s="25" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
         <v>27</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C30" s="22" t="s">
         <v>25</v>
@@ -1768,15 +1765,15 @@
       <c r="G30" s="22"/>
       <c r="H30" s="22"/>
       <c r="I30" s="24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="31" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="31" s="25" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
         <v>27</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C31" s="22" t="s">
         <v>25</v>
@@ -1784,15 +1781,15 @@
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
       <c r="F31" s="23" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G31" s="22"/>
       <c r="H31" s="22"/>
       <c r="I31" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
       <c r="C32" s="9"/>
@@ -1803,97 +1800,97 @@
       <c r="H32" s="9"/>
       <c r="I32" s="11"/>
     </row>
-    <row r="33" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="26" t="s">
-        <v>56</v>
-      </c>
-      <c r="B33" s="26" t="s">
+    <row r="33" s="31" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28" t="s">
+      <c r="C33" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="F33" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="G33" s="27" t="s">
+      <c r="F33" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="H33" s="27"/>
-      <c r="I33" s="29" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="34" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="26" t="s">
+      <c r="H33" s="28"/>
+      <c r="I33" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="26" t="s">
+    </row>
+    <row r="34" s="31" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C34" s="27" t="s">
+      <c r="C34" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="28"/>
-      <c r="E34" s="28"/>
-      <c r="F34" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="G34" s="27"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="29" t="s">
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="G34" s="28"/>
+      <c r="H34" s="28"/>
+      <c r="I34" s="30" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" s="31" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="27" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="35" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="B35" s="26" t="s">
+      <c r="B35" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C35" s="27" t="s">
+      <c r="C35" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="28"/>
-      <c r="E35" s="28"/>
-      <c r="F35" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="G35" s="27" t="s">
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="G35" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="H35" s="27"/>
-      <c r="I35" s="29" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="36" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="B36" s="26" t="s">
+      <c r="H35" s="28"/>
+      <c r="I35" s="30" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="36" s="31" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C36" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="D36" s="28"/>
-      <c r="E36" s="28"/>
-      <c r="F36" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="G36" s="27"/>
-      <c r="H36" s="27"/>
-      <c r="I36" s="29" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C36" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="28"/>
+      <c r="H36" s="28"/>
+      <c r="I36" s="30" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="12"/>
       <c r="B37" s="12"/>
       <c r="C37" s="13"/>
@@ -1904,78 +1901,78 @@
       <c r="H37" s="13"/>
       <c r="I37" s="15"/>
     </row>
-    <row r="38" s="35" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="31" t="s">
+    <row r="38" s="36" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="B38" s="31" t="s">
+      <c r="B38" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C38" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="D38" s="33"/>
-      <c r="E38" s="33" t="s">
+      <c r="C38" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="34"/>
+      <c r="E38" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="F38" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="G38" s="32" t="s">
+      <c r="F38" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="G38" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="H38" s="32"/>
-      <c r="I38" s="34" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="39" s="35" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="31" t="s">
+      <c r="H38" s="33"/>
+      <c r="I38" s="35" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="39" s="36" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="B39" s="31" t="s">
+      <c r="B39" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C39" s="32" t="s">
+      <c r="C39" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="D39" s="33"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="G39" s="32" t="s">
-        <v>49</v>
-      </c>
-      <c r="H39" s="32"/>
-      <c r="I39" s="34" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="40" s="35" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="31" t="s">
+      <c r="D39" s="34"/>
+      <c r="E39" s="34"/>
+      <c r="F39" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="H39" s="33"/>
+      <c r="I39" s="35" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" s="36" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="31" t="s">
+      <c r="B40" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="C40" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="D40" s="33"/>
-      <c r="E40" s="33"/>
-      <c r="F40" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="G40" s="32" t="n">
+      <c r="C40" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="34"/>
+      <c r="E40" s="34"/>
+      <c r="F40" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="H40" s="32"/>
-      <c r="I40" s="34" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H40" s="33"/>
+      <c r="I40" s="37" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="12"/>
       <c r="B41" s="12"/>
       <c r="C41" s="13"/>
@@ -1986,220 +1983,220 @@
       <c r="H41" s="13"/>
       <c r="I41" s="15"/>
     </row>
-    <row r="42" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="36" t="s">
+    <row r="42" s="42" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B42" s="36" t="s">
+      <c r="B42" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="C42" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="D42" s="38"/>
-      <c r="E42" s="38" t="s">
+      <c r="C42" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D42" s="40"/>
+      <c r="E42" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="F42" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="G42" s="37" t="s">
+      <c r="F42" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="G42" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="H42" s="37"/>
-      <c r="I42" s="39" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="43" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="36" t="s">
+      <c r="H42" s="39"/>
+      <c r="I42" s="41" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="43" s="42" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B43" s="36" t="s">
+      <c r="B43" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C43" s="37" t="s">
+      <c r="C43" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="D43" s="38"/>
-      <c r="E43" s="38"/>
-      <c r="F43" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="G43" s="37"/>
-      <c r="H43" s="37"/>
-      <c r="I43" s="39" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="44" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="36" t="s">
+      <c r="D43" s="40"/>
+      <c r="E43" s="40"/>
+      <c r="F43" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="G43" s="39"/>
+      <c r="H43" s="39"/>
+      <c r="I43" s="41" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="44" s="42" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B44" s="36" t="s">
+      <c r="B44" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="C44" s="37" t="s">
+      <c r="C44" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="D44" s="38"/>
-      <c r="E44" s="38"/>
-      <c r="F44" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="G44" s="37"/>
-      <c r="H44" s="37"/>
-      <c r="I44" s="39" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="45" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="36" t="s">
+      <c r="D44" s="40"/>
+      <c r="E44" s="40"/>
+      <c r="F44" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="G44" s="39"/>
+      <c r="H44" s="39"/>
+      <c r="I44" s="41" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="45" s="42" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B45" s="36" t="s">
-        <v>65</v>
-      </c>
-      <c r="C45" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="D45" s="38"/>
-      <c r="E45" s="38" t="s">
+      <c r="B45" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="C45" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="40"/>
+      <c r="E45" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F45" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="G45" s="37"/>
-      <c r="H45" s="37" t="s">
-        <v>66</v>
-      </c>
-      <c r="I45" s="39" t="s">
+      <c r="F45" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="G45" s="39"/>
+      <c r="H45" s="39" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="46" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="36" t="s">
+      <c r="I45" s="41" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="46" s="42" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B46" s="41" t="s">
-        <v>68</v>
-      </c>
-      <c r="C46" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="D46" s="38"/>
-      <c r="E46" s="38" t="s">
+      <c r="B46" s="43" t="s">
+        <v>69</v>
+      </c>
+      <c r="C46" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D46" s="40"/>
+      <c r="E46" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F46" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="G46" s="37"/>
-      <c r="H46" s="37" t="s">
-        <v>69</v>
-      </c>
-      <c r="I46" s="39" t="s">
+      <c r="F46" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="G46" s="39"/>
+      <c r="H46" s="39" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="47" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="36" t="s">
+      <c r="I46" s="41" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="47" s="42" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B47" s="41" t="s">
-        <v>71</v>
-      </c>
-      <c r="C47" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="D47" s="38"/>
-      <c r="E47" s="38" t="s">
+      <c r="B47" s="43" t="s">
+        <v>72</v>
+      </c>
+      <c r="C47" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D47" s="40"/>
+      <c r="E47" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F47" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="G47" s="37"/>
-      <c r="H47" s="37" t="s">
-        <v>72</v>
-      </c>
-      <c r="I47" s="39" t="s">
+      <c r="F47" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="G47" s="39"/>
+      <c r="H47" s="39" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="48" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="36" t="s">
+      <c r="I47" s="41" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="48" s="42" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B48" s="36" t="s">
-        <v>74</v>
-      </c>
-      <c r="C48" s="37" t="s">
+      <c r="B48" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="C48" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="D48" s="38"/>
-      <c r="E48" s="38"/>
-      <c r="F48" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="G48" s="37" t="s">
-        <v>49</v>
-      </c>
-      <c r="H48" s="37"/>
-      <c r="I48" s="39" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="49" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="36" t="s">
+      <c r="D48" s="40"/>
+      <c r="E48" s="40"/>
+      <c r="F48" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="G48" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="H48" s="39"/>
+      <c r="I48" s="41" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="49" s="42" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B49" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="C49" s="37" t="s">
+      <c r="B49" s="38" t="s">
+        <v>77</v>
+      </c>
+      <c r="C49" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="D49" s="38"/>
-      <c r="E49" s="38"/>
-      <c r="F49" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="G49" s="37" t="s">
-        <v>49</v>
-      </c>
-      <c r="H49" s="37"/>
-      <c r="I49" s="39" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="50" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="36" t="s">
+      <c r="D49" s="40"/>
+      <c r="E49" s="40"/>
+      <c r="F49" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="G49" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="H49" s="39"/>
+      <c r="I49" s="41" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="50" s="42" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B50" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="C50" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="D50" s="38"/>
-      <c r="E50" s="38" t="s">
+      <c r="B50" s="38" t="s">
+        <v>79</v>
+      </c>
+      <c r="C50" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D50" s="40"/>
+      <c r="E50" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F50" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="G50" s="37"/>
-      <c r="H50" s="37" t="s">
-        <v>79</v>
-      </c>
-      <c r="I50" s="39" t="s">
+      <c r="F50" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="G50" s="39"/>
+      <c r="H50" s="39" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I50" s="41" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="8"/>
       <c r="B51" s="12"/>
       <c r="C51" s="13"/>
@@ -2210,128 +2207,128 @@
       <c r="H51" s="13"/>
       <c r="I51" s="15"/>
     </row>
-    <row r="52" s="47" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="43" t="s">
-        <v>66</v>
-      </c>
-      <c r="B52" s="43" t="s">
+    <row r="52" s="48" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="44" t="s">
+        <v>67</v>
+      </c>
+      <c r="B52" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="C52" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="D52" s="45"/>
-      <c r="E52" s="45" t="s">
+      <c r="C52" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="D52" s="46"/>
+      <c r="E52" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="F52" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="G52" s="44" t="s">
+      <c r="F52" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="G52" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="H52" s="44"/>
-      <c r="I52" s="46" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="53" s="47" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="43" t="s">
-        <v>66</v>
-      </c>
-      <c r="B53" s="43" t="s">
+      <c r="H52" s="45"/>
+      <c r="I52" s="47" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="53" s="48" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="44" t="s">
+        <v>67</v>
+      </c>
+      <c r="B53" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="C53" s="44" t="s">
+      <c r="C53" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="D53" s="45"/>
-      <c r="E53" s="45"/>
-      <c r="F53" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="G53" s="44" t="s">
-        <v>49</v>
-      </c>
-      <c r="H53" s="44"/>
-      <c r="I53" s="46" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="54" s="47" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="43" t="s">
-        <v>66</v>
-      </c>
-      <c r="B54" s="43" t="s">
+      <c r="D53" s="46"/>
+      <c r="E53" s="46"/>
+      <c r="F53" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="G53" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="H53" s="45"/>
+      <c r="I53" s="47" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="54" s="48" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="44" t="s">
+        <v>67</v>
+      </c>
+      <c r="B54" s="44" t="s">
         <v>41</v>
       </c>
-      <c r="C54" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="D54" s="45"/>
-      <c r="E54" s="45"/>
-      <c r="F54" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="G54" s="44" t="n">
+      <c r="C54" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="D54" s="46"/>
+      <c r="E54" s="46"/>
+      <c r="F54" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="G54" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="H54" s="44"/>
-      <c r="I54" s="46" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="55" s="47" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="43" t="s">
-        <v>66</v>
-      </c>
-      <c r="B55" s="43" t="s">
+      <c r="H54" s="45"/>
+      <c r="I54" s="49" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="55" s="48" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="44" t="s">
+        <v>67</v>
+      </c>
+      <c r="B55" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="C55" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="D55" s="45"/>
-      <c r="E55" s="45" t="s">
+      <c r="C55" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="D55" s="46"/>
+      <c r="E55" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="F55" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="G55" s="44"/>
-      <c r="H55" s="44" t="s">
+      <c r="F55" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="G55" s="45"/>
+      <c r="H55" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="I55" s="46" t="s">
+      <c r="I55" s="47" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="56" s="47" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="43" t="s">
-        <v>66</v>
-      </c>
-      <c r="B56" s="43" t="s">
+    <row r="56" s="48" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="44" t="s">
+        <v>67</v>
+      </c>
+      <c r="B56" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="C56" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="D56" s="45"/>
-      <c r="E56" s="45" t="s">
+      <c r="C56" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="D56" s="46"/>
+      <c r="E56" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="F56" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="G56" s="44"/>
-      <c r="H56" s="44" t="s">
+      <c r="F56" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="G56" s="45"/>
+      <c r="H56" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="I56" s="46" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I56" s="47" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="8"/>
       <c r="B57" s="8"/>
       <c r="C57" s="9"/>
@@ -2342,128 +2339,128 @@
       <c r="H57" s="9"/>
       <c r="I57" s="11"/>
     </row>
-    <row r="58" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="48" t="s">
-        <v>69</v>
-      </c>
-      <c r="B58" s="48" t="s">
+    <row r="58" s="54" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="B58" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="C58" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="D58" s="50"/>
-      <c r="E58" s="50" t="s">
+      <c r="C58" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="D58" s="52"/>
+      <c r="E58" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="F58" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="G58" s="49" t="s">
+      <c r="F58" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G58" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="H58" s="49"/>
-      <c r="I58" s="51" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="59" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="48" t="s">
-        <v>69</v>
-      </c>
-      <c r="B59" s="48" t="s">
+      <c r="H58" s="51"/>
+      <c r="I58" s="53" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="59" s="54" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="B59" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="C59" s="49" t="s">
+      <c r="C59" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="D59" s="50"/>
-      <c r="E59" s="50"/>
-      <c r="F59" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="G59" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="H59" s="49"/>
-      <c r="I59" s="51" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="60" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="48" t="s">
-        <v>69</v>
-      </c>
-      <c r="B60" s="48" t="s">
+      <c r="D59" s="52"/>
+      <c r="E59" s="52"/>
+      <c r="F59" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G59" s="51" t="s">
+        <v>50</v>
+      </c>
+      <c r="H59" s="51"/>
+      <c r="I59" s="53" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="60" s="54" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="B60" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="C60" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="D60" s="50"/>
-      <c r="E60" s="50"/>
-      <c r="F60" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="G60" s="49" t="n">
+      <c r="C60" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="D60" s="52"/>
+      <c r="E60" s="52"/>
+      <c r="F60" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G60" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="H60" s="49"/>
-      <c r="I60" s="51" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="61" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="48" t="s">
-        <v>69</v>
-      </c>
-      <c r="B61" s="48" t="s">
+      <c r="H60" s="51"/>
+      <c r="I60" s="55" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="61" s="54" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="B61" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="C61" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="D61" s="50"/>
-      <c r="E61" s="50" t="s">
+      <c r="C61" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="D61" s="52"/>
+      <c r="E61" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="F61" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="G61" s="49"/>
-      <c r="H61" s="49" t="s">
+      <c r="F61" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G61" s="51"/>
+      <c r="H61" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="I61" s="51" t="s">
+      <c r="I61" s="53" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="62" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="48" t="s">
-        <v>69</v>
-      </c>
-      <c r="B62" s="48" t="s">
+    <row r="62" s="54" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="B62" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="C62" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="D62" s="50"/>
-      <c r="E62" s="50" t="s">
+      <c r="C62" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="D62" s="52"/>
+      <c r="E62" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="F62" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="G62" s="49"/>
-      <c r="H62" s="49" t="s">
+      <c r="F62" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G62" s="51"/>
+      <c r="H62" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="I62" s="51" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I62" s="53" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="8"/>
       <c r="B63" s="8"/>
       <c r="C63" s="9"/>
@@ -2474,128 +2471,128 @@
       <c r="H63" s="9"/>
       <c r="I63" s="11"/>
     </row>
-    <row r="64" s="57" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="53" t="s">
-        <v>72</v>
-      </c>
-      <c r="B64" s="53" t="s">
+    <row r="64" s="60" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="56" t="s">
+        <v>73</v>
+      </c>
+      <c r="B64" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="C64" s="54" t="s">
-        <v>19</v>
-      </c>
-      <c r="D64" s="55"/>
-      <c r="E64" s="55" t="s">
+      <c r="C64" s="57" t="s">
+        <v>19</v>
+      </c>
+      <c r="D64" s="58"/>
+      <c r="E64" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="F64" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="G64" s="54" t="s">
+      <c r="F64" s="58" t="s">
+        <v>21</v>
+      </c>
+      <c r="G64" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="H64" s="54"/>
-      <c r="I64" s="56" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="65" s="57" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="53" t="s">
-        <v>72</v>
-      </c>
-      <c r="B65" s="53" t="s">
+      <c r="H64" s="57"/>
+      <c r="I64" s="59" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="65" s="60" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="56" t="s">
+        <v>73</v>
+      </c>
+      <c r="B65" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="C65" s="54" t="s">
+      <c r="C65" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="D65" s="55"/>
-      <c r="E65" s="55"/>
-      <c r="F65" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="G65" s="54" t="s">
-        <v>49</v>
-      </c>
-      <c r="H65" s="54"/>
-      <c r="I65" s="56" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="66" s="57" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="53" t="s">
-        <v>72</v>
-      </c>
-      <c r="B66" s="53" t="s">
+      <c r="D65" s="58"/>
+      <c r="E65" s="58"/>
+      <c r="F65" s="58" t="s">
+        <v>21</v>
+      </c>
+      <c r="G65" s="57" t="s">
+        <v>50</v>
+      </c>
+      <c r="H65" s="57"/>
+      <c r="I65" s="59" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" s="60" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="56" t="s">
+        <v>73</v>
+      </c>
+      <c r="B66" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="C66" s="54" t="s">
-        <v>19</v>
-      </c>
-      <c r="D66" s="55"/>
-      <c r="E66" s="55"/>
-      <c r="F66" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="G66" s="54" t="n">
+      <c r="C66" s="57" t="s">
+        <v>19</v>
+      </c>
+      <c r="D66" s="58"/>
+      <c r="E66" s="58"/>
+      <c r="F66" s="58" t="s">
+        <v>21</v>
+      </c>
+      <c r="G66" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="H66" s="54"/>
-      <c r="I66" s="56" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="67" s="57" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="53" t="s">
-        <v>72</v>
-      </c>
-      <c r="B67" s="53" t="s">
+      <c r="H66" s="57"/>
+      <c r="I66" s="61" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="67" s="60" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="56" t="s">
+        <v>73</v>
+      </c>
+      <c r="B67" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="C67" s="54" t="s">
-        <v>19</v>
-      </c>
-      <c r="D67" s="55"/>
-      <c r="E67" s="55" t="s">
+      <c r="C67" s="57" t="s">
+        <v>19</v>
+      </c>
+      <c r="D67" s="58"/>
+      <c r="E67" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="F67" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="G67" s="54"/>
-      <c r="H67" s="54" t="s">
+      <c r="F67" s="58" t="s">
+        <v>21</v>
+      </c>
+      <c r="G67" s="57"/>
+      <c r="H67" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="I67" s="56" t="s">
+      <c r="I67" s="59" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="68" s="57" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="53" t="s">
-        <v>72</v>
-      </c>
-      <c r="B68" s="53" t="s">
+    <row r="68" s="60" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="56" t="s">
+        <v>73</v>
+      </c>
+      <c r="B68" s="56" t="s">
         <v>45</v>
       </c>
-      <c r="C68" s="54" t="s">
-        <v>19</v>
-      </c>
-      <c r="D68" s="55"/>
-      <c r="E68" s="55" t="s">
+      <c r="C68" s="57" t="s">
+        <v>19</v>
+      </c>
+      <c r="D68" s="58"/>
+      <c r="E68" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="F68" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="G68" s="54"/>
-      <c r="H68" s="54" t="s">
+      <c r="F68" s="58" t="s">
+        <v>21</v>
+      </c>
+      <c r="G68" s="57"/>
+      <c r="H68" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="I68" s="56" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I68" s="59" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="8"/>
       <c r="B69" s="8"/>
       <c r="C69" s="9"/>
@@ -2606,50 +2603,274 @@
       <c r="H69" s="9"/>
       <c r="I69" s="11"/>
     </row>
-    <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="12"/>
-      <c r="B70" s="12"/>
-      <c r="C70" s="13"/>
-      <c r="D70" s="14"/>
-      <c r="E70" s="14"/>
-      <c r="F70" s="14"/>
-      <c r="G70" s="13"/>
+      <c r="B70" s="62" t="s">
+        <v>88</v>
+      </c>
+      <c r="C70" s="62" t="s">
+        <v>89</v>
+      </c>
+      <c r="D70" s="62" t="s">
+        <v>90</v>
+      </c>
+      <c r="E70" s="62" t="s">
+        <v>91</v>
+      </c>
+      <c r="F70" s="62" t="s">
+        <v>92</v>
+      </c>
+      <c r="G70" s="62" t="s">
+        <v>93</v>
+      </c>
       <c r="H70" s="13"/>
       <c r="I70" s="15"/>
     </row>
-    <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="8"/>
-      <c r="B71" s="8"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="10"/>
-      <c r="E71" s="10"/>
-      <c r="F71" s="10"/>
-      <c r="G71" s="9"/>
-      <c r="H71" s="9"/>
-      <c r="I71" s="11"/>
-    </row>
-    <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="12"/>
-      <c r="B72" s="12"/>
-      <c r="C72" s="13"/>
-      <c r="D72" s="14"/>
-      <c r="E72" s="14"/>
-      <c r="F72" s="14"/>
-      <c r="G72" s="13"/>
-      <c r="H72" s="13"/>
-      <c r="I72" s="15"/>
+    <row r="71" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B71" s="63" t="s">
+        <v>18</v>
+      </c>
+      <c r="C71" s="64" t="s">
+        <v>19</v>
+      </c>
+      <c r="D71" s="64"/>
+      <c r="E71" s="64" t="s">
+        <v>20</v>
+      </c>
+      <c r="F71" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="G71" s="64" t="s">
+        <v>22</v>
+      </c>
+      <c r="H71" s="64"/>
+    </row>
+    <row r="72" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B72" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="C72" s="64" t="s">
+        <v>19</v>
+      </c>
+      <c r="D72" s="64"/>
+      <c r="E72" s="64" t="s">
+        <v>37</v>
+      </c>
+      <c r="F72" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="G72" s="64"/>
+      <c r="H72" s="64" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="73" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B73" s="63" t="s">
+        <v>97</v>
+      </c>
+      <c r="C73" s="64" t="s">
+        <v>19</v>
+      </c>
+      <c r="D73" s="64"/>
+      <c r="E73" s="64" t="s">
+        <v>37</v>
+      </c>
+      <c r="F73" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="G73" s="64"/>
+      <c r="H73" s="64" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="74" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B74" s="63" t="s">
+        <v>99</v>
+      </c>
+      <c r="C74" s="64" t="s">
+        <v>19</v>
+      </c>
+      <c r="D74" s="64"/>
+      <c r="E74" s="64" t="s">
+        <v>37</v>
+      </c>
+      <c r="F74" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="G74" s="64"/>
+      <c r="H74" s="64" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="75" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B75" s="63" t="s">
+        <v>101</v>
+      </c>
+      <c r="C75" s="64" t="s">
+        <v>25</v>
+      </c>
+      <c r="D75" s="64"/>
+      <c r="E75" s="64"/>
+      <c r="F75" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="G75" s="64" t="s">
+        <v>102</v>
+      </c>
+      <c r="H75" s="64" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="76" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B76" s="63" t="s">
+        <v>104</v>
+      </c>
+      <c r="C76" s="64" t="s">
+        <v>25</v>
+      </c>
+      <c r="D76" s="64"/>
+      <c r="E76" s="64"/>
+      <c r="F76" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="G76" s="64"/>
+      <c r="H76" s="64" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="77" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B77" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="C77" s="64" t="s">
+        <v>25</v>
+      </c>
+      <c r="D77" s="64"/>
+      <c r="E77" s="64"/>
+      <c r="F77" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="G77" s="64"/>
+      <c r="H77" s="64" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="78" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B78" s="63" t="s">
+        <v>106</v>
+      </c>
+      <c r="C78" s="64" t="s">
+        <v>25</v>
+      </c>
+      <c r="D78" s="64"/>
+      <c r="E78" s="64"/>
+      <c r="F78" s="65" t="s">
+        <v>55</v>
+      </c>
+      <c r="G78" s="64"/>
+      <c r="H78" s="64" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="79" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B79" s="63" t="s">
+        <v>107</v>
+      </c>
+      <c r="C79" s="64" t="s">
+        <v>25</v>
+      </c>
+      <c r="D79" s="64"/>
+      <c r="E79" s="64" t="s">
+        <v>37</v>
+      </c>
+      <c r="F79" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="G79" s="64"/>
+      <c r="H79" s="64" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="80" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B80" s="63" t="s">
+        <v>109</v>
+      </c>
+      <c r="C80" s="64" t="s">
+        <v>19</v>
+      </c>
+      <c r="D80" s="64"/>
+      <c r="E80" s="64"/>
+      <c r="F80" s="65" t="s">
+        <v>55</v>
+      </c>
+      <c r="G80" s="64"/>
+      <c r="H80" s="64" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="81" s="63" customFormat="true" ht="25.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="B81" s="63" t="s">
+        <v>110</v>
+      </c>
+      <c r="C81" s="64" t="s">
+        <v>19</v>
+      </c>
+      <c r="D81" s="64"/>
+      <c r="E81" s="64" t="s">
+        <v>37</v>
+      </c>
+      <c r="F81" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="G81" s="64"/>
+      <c r="H81" s="64" t="s">
+        <v>98</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C15 C17:C72" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C15 C17:C69" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E15 E17:E72" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E15 E17:E69" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F15 F17:F72" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F15 F17:F69 F71:F81" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2684,97 +2905,100 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="58" t="s">
-        <v>89</v>
-      </c>
-      <c r="B4" s="59" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="58" t="s">
-        <v>91</v>
-      </c>
-      <c r="B5" s="59" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="58" t="s">
-        <v>93</v>
-      </c>
-      <c r="B6" s="59" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="B7" s="59" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="58" t="s">
-        <v>97</v>
-      </c>
-      <c r="B8" s="59" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="58" t="s">
-        <v>99</v>
-      </c>
-      <c r="B9" s="59" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="58" t="s">
-        <v>101</v>
-      </c>
-      <c r="B10" s="59" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="58" t="s">
-        <v>103</v>
-      </c>
-      <c r="B11" s="59" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="58" t="s">
-        <v>105</v>
-      </c>
-      <c r="B12" s="59" t="s">
-        <v>106</v>
-      </c>
-    </row>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="66" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="67" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="66" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" s="67" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="66" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" s="67" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="66" t="s">
+        <v>119</v>
+      </c>
+      <c r="B7" s="67" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="66" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" s="67" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="66" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" s="67" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="66" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" s="67" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="66" t="s">
+        <v>127</v>
+      </c>
+      <c r="B11" s="67" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="66" t="s">
+        <v>129</v>
+      </c>
+      <c r="B12" s="67" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="60" t="s">
-        <v>107</v>
-      </c>
-    </row>
+      <c r="A14" s="68" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
         <v>8</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>108</v>
+        <v>132</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>10</v>
@@ -2789,10 +3013,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>16</v>
@@ -2800,16 +3024,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>20</v>
@@ -2818,131 +3042,131 @@
         <v>21</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="H17" s="12" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>21</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>21</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>122</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>123</v>
+        <v>147</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>21</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>37</v>
@@ -2951,27 +3175,27 @@
         <v>21</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>131</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>20</v>
@@ -2980,65 +3204,65 @@
         <v>21</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="F24" s="10" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -3058,9 +3282,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -3068,12 +3292,12 @@
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>37</v>
@@ -3082,55 +3306,55 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>149</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>